<commit_message>
Cleaned up the mess in scenarios. Fixed the readme
</commit_message>
<xml_diff>
--- a/scenario_tiers.xlsx
+++ b/scenario_tiers.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PhD\Research\Norma\Code\norma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B1B096D-8AD4-4A11-9B3C-2345C07C0931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EBDA2CA-161E-42D3-8A68-9B48B4DB3050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="218">
   <si>
     <t>Goal</t>
   </si>
@@ -684,6 +684,9 @@
   </si>
   <si>
     <t>N0, N21, N19, N20</t>
+  </si>
+  <si>
+    <t>Goal Label</t>
   </si>
 </sst>
 </file>
@@ -745,15 +748,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5531204B-3ED6-4CA8-89E2-82AEC7F0A652}" name="Curated_Benchmark" displayName="Curated_Benchmark" ref="A1:F56" totalsRowShown="0">
-  <autoFilter ref="A1:F56" xr:uid="{5531204B-3ED6-4CA8-89E2-82AEC7F0A652}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5531204B-3ED6-4CA8-89E2-82AEC7F0A652}" name="Curated_Benchmark" displayName="Curated_Benchmark" ref="A1:G57" totalsRowCount="1">
+  <autoFilter ref="A1:G56" xr:uid="{5531204B-3ED6-4CA8-89E2-82AEC7F0A652}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{6FA642A6-7341-46EA-9E06-98E22C1B3E7B}" name="ID"/>
     <tableColumn id="2" xr3:uid="{709CB8AB-30D5-4DF7-ABDE-37DF3A858485}" name="Title"/>
     <tableColumn id="3" xr3:uid="{F50FEE1D-6841-4853-A67F-A3A304F3C06F}" name="Norms"/>
     <tableColumn id="4" xr3:uid="{1D648367-56F0-4647-9057-A4B5AF6E4CD5}" name="Goal"/>
     <tableColumn id="5" xr3:uid="{77FE9F44-B02B-492C-996F-BF8C822C342D}" name="Sanctions"/>
     <tableColumn id="6" xr3:uid="{F21937A1-E693-4BFA-A0F6-E2E58404BCB8}" name="Label"/>
+    <tableColumn id="7" xr3:uid="{C29735F7-8BFE-457C-8B34-384557BD9390}" name="Goal Label" totalsRowFunction="custom">
+      <totalsRowFormula>AVERAGE(G2:G51)</totalsRowFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1044,7 +1050,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6431D2D6-02C3-4DB1-9FF6-4BAA3309EB58}">
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="26.36328125" bestFit="1" customWidth="1"/>
@@ -1074,6 +1080,9 @@
       <c r="F1" t="s">
         <v>136</v>
       </c>
+      <c r="G1" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -1094,12 +1103,15 @@
       <c r="F2" t="s">
         <v>164</v>
       </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
       <c r="H2" t="s">
         <v>138</v>
       </c>
       <c r="I2">
         <f>COUNTIF(F:F, "*Conflict*")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J2" t="s">
         <v>161</v>
@@ -1124,12 +1136,15 @@
       <c r="F3" t="s">
         <v>139</v>
       </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
       <c r="H3" t="s">
         <v>164</v>
       </c>
       <c r="I3">
         <f>COUNTIF(F:F, "*Delayed*")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J3" t="s">
         <v>162</v>
@@ -1154,6 +1169,9 @@
       <c r="F4" t="s">
         <v>164</v>
       </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
       <c r="H4" t="s">
         <v>139</v>
       </c>
@@ -1184,6 +1202,9 @@
       <c r="F5" t="s">
         <v>164</v>
       </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
       <c r="H5" t="s">
         <v>213</v>
       </c>
@@ -1211,6 +1232,9 @@
       <c r="F6" t="s">
         <v>164</v>
       </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1229,7 +1253,10 @@
         <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>138</v>
+        <v>164</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -1251,6 +1278,9 @@
       <c r="F8" t="s">
         <v>164</v>
       </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1271,6 +1301,9 @@
       <c r="F9" t="s">
         <v>164</v>
       </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1291,6 +1324,9 @@
       <c r="F10" t="s">
         <v>139</v>
       </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1311,6 +1347,9 @@
       <c r="F11" t="s">
         <v>138</v>
       </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1331,6 +1370,9 @@
       <c r="F12" t="s">
         <v>164</v>
       </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1351,6 +1393,9 @@
       <c r="F13" t="s">
         <v>164</v>
       </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1371,6 +1416,9 @@
       <c r="F14" t="s">
         <v>164</v>
       </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1391,6 +1439,9 @@
       <c r="F15" t="s">
         <v>138</v>
       </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1411,8 +1462,11 @@
       <c r="F16" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>100</v>
       </c>
@@ -1431,8 +1485,11 @@
       <c r="F17" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>101</v>
       </c>
@@ -1451,8 +1508,11 @@
       <c r="F18" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>102</v>
       </c>
@@ -1471,8 +1531,11 @@
       <c r="F19" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>103</v>
       </c>
@@ -1491,8 +1554,11 @@
       <c r="F20" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>104</v>
       </c>
@@ -1511,8 +1577,11 @@
       <c r="F21" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>105</v>
       </c>
@@ -1531,8 +1600,11 @@
       <c r="F22" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>106</v>
       </c>
@@ -1551,8 +1623,11 @@
       <c r="F23" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>107</v>
       </c>
@@ -1571,8 +1646,11 @@
       <c r="F24" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>108</v>
       </c>
@@ -1591,8 +1669,11 @@
       <c r="F25" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>109</v>
       </c>
@@ -1611,8 +1692,11 @@
       <c r="F26" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>110</v>
       </c>
@@ -1631,8 +1715,11 @@
       <c r="F27" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>111</v>
       </c>
@@ -1651,8 +1738,11 @@
       <c r="F28" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>112</v>
       </c>
@@ -1671,8 +1761,11 @@
       <c r="F29" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>113</v>
       </c>
@@ -1691,8 +1784,11 @@
       <c r="F30" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>114</v>
       </c>
@@ -1711,8 +1807,11 @@
       <c r="F31" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>115</v>
       </c>
@@ -1731,8 +1830,11 @@
       <c r="F32" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>116</v>
       </c>
@@ -1751,8 +1853,11 @@
       <c r="F33" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>117</v>
       </c>
@@ -1771,8 +1876,11 @@
       <c r="F34" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>118</v>
       </c>
@@ -1791,8 +1899,11 @@
       <c r="F35" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>119</v>
       </c>
@@ -1811,8 +1922,11 @@
       <c r="F36" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>120</v>
       </c>
@@ -1831,8 +1945,11 @@
       <c r="F37" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>121</v>
       </c>
@@ -1851,8 +1968,11 @@
       <c r="F38" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>122</v>
       </c>
@@ -1871,8 +1991,11 @@
       <c r="F39" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>123</v>
       </c>
@@ -1891,8 +2014,11 @@
       <c r="F40" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>124</v>
       </c>
@@ -1911,8 +2037,11 @@
       <c r="F41" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>125</v>
       </c>
@@ -1931,8 +2060,11 @@
       <c r="F42" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>126</v>
       </c>
@@ -1951,8 +2083,11 @@
       <c r="F43" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>127</v>
       </c>
@@ -1971,8 +2106,11 @@
       <c r="F44" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>128</v>
       </c>
@@ -1991,8 +2129,11 @@
       <c r="F45" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>129</v>
       </c>
@@ -2011,8 +2152,11 @@
       <c r="F46" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>130</v>
       </c>
@@ -2031,8 +2175,11 @@
       <c r="F47" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>131</v>
       </c>
@@ -2051,8 +2198,11 @@
       <c r="F48" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>132</v>
       </c>
@@ -2071,8 +2221,11 @@
       <c r="F49" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>133</v>
       </c>
@@ -2091,8 +2244,11 @@
       <c r="F50" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>134</v>
       </c>
@@ -2111,8 +2267,11 @@
       <c r="F51" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>198</v>
       </c>
@@ -2131,8 +2290,11 @@
       <c r="F52" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>199</v>
       </c>
@@ -2151,8 +2313,11 @@
       <c r="F53" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>200</v>
       </c>
@@ -2171,8 +2336,11 @@
       <c r="F54" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>201</v>
       </c>
@@ -2191,8 +2359,11 @@
       <c r="F55" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G55">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>202</v>
       </c>
@@ -2210,6 +2381,15 @@
       </c>
       <c r="F56" t="s">
         <v>212</v>
+      </c>
+      <c r="G56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G57">
+        <f>AVERAGE(G2:G51)</f>
+        <v>0.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>